<commit_message>
Test Plan 2, Test Report 2, spreadsheet update
Test Plan 2 and Test Report 2 uploaded. Also, spreadsheet got a date or two.
</commit_message>
<xml_diff>
--- a/project requirements spreadsheet.xlsx
+++ b/project requirements spreadsheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/soapmac/Documents/GitHub/Shattered-Protocols-Text-RPG/Shattered Protocols/Shattered-Protocols-Text-RPG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA6583C0-B331-9C44-9289-C2D774B87B6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{535770FE-49E1-1C41-AD7D-F26A1B45554D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15820" xr2:uid="{CAB5D44A-E176-404C-B398-BEAD2D9E6884}"/>
   </bookViews>
@@ -940,47 +940,47 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="13" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1341,52 +1341,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="27" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="83" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="90"/>
+      <c r="B1" s="84"/>
       <c r="C1" s="25"/>
-      <c r="D1" s="95" t="s">
+      <c r="D1" s="90" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
-      <c r="I1" s="95"/>
-      <c r="J1" s="95"/>
-      <c r="K1" s="95"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
       <c r="L1" s="25"/>
       <c r="M1" s="67"/>
     </row>
     <row r="2" spans="1:13" s="27" customFormat="1" ht="19" x14ac:dyDescent="0.2">
-      <c r="A2" s="91" t="s">
+      <c r="A2" s="85" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="92"/>
+      <c r="B2" s="86"/>
       <c r="C2" s="25"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
-      <c r="I2" s="95"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="95"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="90"/>
+      <c r="G2" s="90"/>
+      <c r="H2" s="90"/>
+      <c r="I2" s="90"/>
+      <c r="J2" s="90"/>
+      <c r="K2" s="90"/>
       <c r="M2" s="68"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="42"/>
       <c r="B3" s="30"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="95"/>
-      <c r="E3" s="95"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="95"/>
-      <c r="H3" s="95"/>
-      <c r="I3" s="95"/>
-      <c r="J3" s="95"/>
-      <c r="K3" s="95"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
       <c r="L3" s="13"/>
       <c r="M3" s="69"/>
     </row>
@@ -1397,14 +1397,14 @@
       <c r="B4" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="95"/>
-      <c r="H4" s="95"/>
-      <c r="I4" s="95"/>
-      <c r="J4" s="95"/>
-      <c r="K4" s="95"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="90"/>
+      <c r="F4" s="90"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="90"/>
       <c r="M4" s="70"/>
     </row>
     <row r="5" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.2">
@@ -1414,14 +1414,14 @@
       <c r="B5" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="95"/>
-      <c r="E5" s="95"/>
-      <c r="F5" s="95"/>
-      <c r="G5" s="95"/>
-      <c r="H5" s="95"/>
-      <c r="I5" s="95"/>
-      <c r="J5" s="95"/>
-      <c r="K5" s="95"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="90"/>
+      <c r="F5" s="90"/>
+      <c r="G5" s="90"/>
+      <c r="H5" s="90"/>
+      <c r="I5" s="90"/>
+      <c r="J5" s="90"/>
+      <c r="K5" s="90"/>
       <c r="M5" s="70"/>
     </row>
     <row r="6" spans="1:13" s="7" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -1431,14 +1431,14 @@
       <c r="B6" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="D6" s="95"/>
-      <c r="E6" s="95"/>
-      <c r="F6" s="95"/>
-      <c r="G6" s="95"/>
-      <c r="H6" s="95"/>
-      <c r="I6" s="95"/>
-      <c r="J6" s="95"/>
-      <c r="K6" s="95"/>
+      <c r="D6" s="90"/>
+      <c r="E6" s="90"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="90"/>
+      <c r="H6" s="90"/>
+      <c r="I6" s="90"/>
+      <c r="J6" s="90"/>
+      <c r="K6" s="90"/>
       <c r="L6" s="1"/>
       <c r="M6" s="71"/>
     </row>
@@ -1458,73 +1458,73 @@
       <c r="M7" s="71"/>
     </row>
     <row r="8" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="86" t="s">
+      <c r="A8" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="86"/>
-      <c r="C8" s="86"/>
-      <c r="D8" s="86"/>
-      <c r="E8" s="86"/>
-      <c r="F8" s="86"/>
-      <c r="G8" s="86"/>
-      <c r="H8" s="86"/>
-      <c r="I8" s="86"/>
-      <c r="J8" s="86"/>
-      <c r="K8" s="86"/>
-      <c r="L8" s="86"/>
-      <c r="M8" s="86"/>
+      <c r="B8" s="91"/>
+      <c r="C8" s="91"/>
+      <c r="D8" s="91"/>
+      <c r="E8" s="91"/>
+      <c r="F8" s="91"/>
+      <c r="G8" s="91"/>
+      <c r="H8" s="91"/>
+      <c r="I8" s="91"/>
+      <c r="J8" s="91"/>
+      <c r="K8" s="91"/>
+      <c r="L8" s="91"/>
+      <c r="M8" s="91"/>
     </row>
     <row r="9" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
       <c r="B9" s="2"/>
-      <c r="C9" s="86" t="s">
+      <c r="C9" s="91" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="86"/>
-      <c r="E9" s="86"/>
-      <c r="F9" s="86"/>
+      <c r="D9" s="91"/>
+      <c r="E9" s="91"/>
+      <c r="F9" s="91"/>
       <c r="G9" s="1"/>
-      <c r="H9" s="86" t="s">
+      <c r="H9" s="91" t="s">
         <v>7</v>
       </c>
-      <c r="I9" s="86"/>
-      <c r="J9" s="86"/>
-      <c r="K9" s="86"/>
-      <c r="L9" s="96" t="s">
+      <c r="I9" s="91"/>
+      <c r="J9" s="91"/>
+      <c r="K9" s="91"/>
+      <c r="L9" s="92" t="s">
         <v>20</v>
       </c>
-      <c r="M9" s="83" t="s">
+      <c r="M9" s="93" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:13" s="7" customFormat="1" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="2"/>
-      <c r="C10" s="85" t="s">
+      <c r="C10" s="89" t="s">
         <v>21</v>
       </c>
       <c r="D10" s="1"/>
-      <c r="E10" s="85" t="s">
+      <c r="E10" s="89" t="s">
         <v>58</v>
       </c>
-      <c r="F10" s="85" t="s">
+      <c r="F10" s="89" t="s">
         <v>59</v>
       </c>
-      <c r="G10" s="85" t="s">
+      <c r="G10" s="89" t="s">
         <v>60</v>
       </c>
-      <c r="H10" s="85" t="s">
+      <c r="H10" s="89" t="s">
         <v>4</v>
       </c>
-      <c r="I10" s="85" t="s">
+      <c r="I10" s="89" t="s">
         <v>21</v>
       </c>
-      <c r="J10" s="85" t="s">
+      <c r="J10" s="89" t="s">
         <v>5</v>
       </c>
       <c r="K10" s="1"/>
-      <c r="L10" s="96"/>
-      <c r="M10" s="83"/>
+      <c r="L10" s="92"/>
+      <c r="M10" s="93"/>
     </row>
     <row r="11" spans="1:13" s="7" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -1533,24 +1533,24 @@
       <c r="B11" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="85"/>
+      <c r="C11" s="89"/>
       <c r="D11" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="85"/>
-      <c r="F11" s="85"/>
-      <c r="G11" s="85"/>
-      <c r="H11" s="85"/>
-      <c r="I11" s="85"/>
-      <c r="J11" s="85"/>
+      <c r="E11" s="89"/>
+      <c r="F11" s="89"/>
+      <c r="G11" s="89"/>
+      <c r="H11" s="89"/>
+      <c r="I11" s="89"/>
+      <c r="J11" s="89"/>
       <c r="K11" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="L11" s="96"/>
-      <c r="M11" s="83"/>
+      <c r="L11" s="92"/>
+      <c r="M11" s="93"/>
     </row>
     <row r="12" spans="1:13" s="57" customFormat="1" ht="51" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="93" t="s">
+      <c r="A12" s="87" t="s">
         <v>40</v>
       </c>
       <c r="B12" s="53"/>
@@ -1577,7 +1577,7 @@
       <c r="M12" s="72"/>
     </row>
     <row r="13" spans="1:13" s="3" customFormat="1" ht="61.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="94"/>
+      <c r="A13" s="88"/>
       <c r="B13" s="8"/>
       <c r="C13" s="10"/>
       <c r="D13" s="10" t="s">
@@ -2192,7 +2192,7 @@
         <v>97</v>
       </c>
       <c r="L35" s="12"/>
-      <c r="M35" s="87" t="s">
+      <c r="M35" s="95" t="s">
         <v>78</v>
       </c>
     </row>
@@ -2224,7 +2224,7 @@
         <v>97</v>
       </c>
       <c r="L36" s="12"/>
-      <c r="M36" s="88"/>
+      <c r="M36" s="96"/>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="50">
@@ -2254,7 +2254,7 @@
         <v>97</v>
       </c>
       <c r="L37" s="12"/>
-      <c r="M37" s="88"/>
+      <c r="M37" s="96"/>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="50">
@@ -2284,7 +2284,7 @@
         <v>97</v>
       </c>
       <c r="L38" s="12"/>
-      <c r="M38" s="88"/>
+      <c r="M38" s="96"/>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="50">
@@ -2314,7 +2314,7 @@
         <v>97</v>
       </c>
       <c r="L39" s="12"/>
-      <c r="M39" s="88"/>
+      <c r="M39" s="96"/>
     </row>
     <row r="40" spans="1:13" ht="32" x14ac:dyDescent="0.2">
       <c r="A40" s="50">
@@ -2832,9 +2832,12 @@
       <c r="E57" s="40">
         <v>45603</v>
       </c>
+      <c r="F57" s="12">
+        <v>45600</v>
+      </c>
       <c r="G57" s="6">
         <f>IF(B57="","",IF(AND(E57&gt;0,F57&gt;0),F57-E57,0))</f>
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="L57" s="12"/>
       <c r="M57" s="75" t="s">
@@ -2970,11 +2973,11 @@
         <f t="shared" ref="D62:D124" si="6">IF(B62="","",D61)</f>
         <v>2</v>
       </c>
-      <c r="E62" s="84" t="s">
+      <c r="E62" s="94" t="s">
         <v>83</v>
       </c>
-      <c r="F62" s="84"/>
-      <c r="G62" s="84"/>
+      <c r="F62" s="94"/>
+      <c r="G62" s="94"/>
       <c r="H62" s="6" t="s">
         <v>97</v>
       </c>
@@ -3176,11 +3179,11 @@
         <f>IF(B69="","",D68)</f>
         <v>2</v>
       </c>
-      <c r="E69" s="84" t="s">
+      <c r="E69" s="94" t="s">
         <v>120</v>
       </c>
-      <c r="F69" s="84"/>
-      <c r="G69" s="84"/>
+      <c r="F69" s="94"/>
+      <c r="G69" s="94"/>
       <c r="L69" s="12">
         <f>IF(B69="","",IF(D69=D68,L68,IF(F69&gt;0,F69,"Not Delivered")))</f>
         <v>0</v>
@@ -3294,9 +3297,12 @@
       <c r="E73" s="40">
         <v>45607</v>
       </c>
+      <c r="F73" s="12">
+        <v>45610</v>
+      </c>
       <c r="G73" s="6">
         <f>IF(B73="","",IF(AND(E73&gt;0,F73&gt;0),F73-E73,0))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L73" s="12"/>
       <c r="M73" s="75" t="s">
@@ -5439,6 +5445,12 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="M35:M39"/>
+    <mergeCell ref="E62:G62"/>
+    <mergeCell ref="E69:G69"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="H9:K9"/>
+    <mergeCell ref="J10:J11"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A12:A13"/>
@@ -5452,12 +5464,6 @@
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="M9:M11"/>
-    <mergeCell ref="E62:G62"/>
-    <mergeCell ref="E69:G69"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="H9:K9"/>
-    <mergeCell ref="J10:J11"/>
-    <mergeCell ref="M35:M39"/>
   </mergeCells>
   <conditionalFormatting sqref="G10:G61 G63:G68 G70:G1048576">
     <cfRule type="colorScale" priority="1">

</xml_diff>